<commit_message>
Auto commit (2026-08-21 19:46) — 1 changes
Claude Code 세션 종료 시 자동 커밋.

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/projects/18_while_my_wifes_away/18_while_my_wifes_away_w3_writer_table_actions.xlsx
+++ b/projects/18_while_my_wifes_away/18_while_my_wifes_away_w3_writer_table_actions.xlsx
@@ -7,11 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="작가 트리트먼트 + 처리" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="원칙 · 계수" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="작가 안내 — 심리 묘사" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="작가 트리트먼트 + 처리" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="원칙 · 계수" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'작가 트리트먼트 + 처리'!$A$1:$F$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'작가 트리트먼트 + 처리'!$A$1:$F$51</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -117,7 +118,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -147,6 +148,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -514,6 +518,314 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="122" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="96" customHeight="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>■ 왜 두 사람의 속마음을 여는가</t>
+        </is>
+      </c>
+      <c r="B1" s="9" t="inlineStr"/>
+    </row>
+    <row r="2" ht="96" customHeight="1">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>결론</t>
+        </is>
+      </c>
+      <c r="B2" s="9" t="inlineStr">
+        <is>
+          <t>다이앤과 콜, 두 사람의 속마음(VO·감각 묘사)을 전면 개방합니다. 기존 기획안의 '다이앤 속마음 폐쇄' 조항은 이번 라운드로 해제합니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="96" customHeight="1">
+      <c r="A3" s="10" t="inlineStr">
+        <is>
+          <t>이유 — 분량 엔진</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>성행위만으로 50화를 채울 수 없습니다. 현재 원고가 그 증거입니다 — 행위 사다리(명령/복종 → 근접자 위험 → 장소 변경 → 사정 통제)가 16화에서 천장을 치고, 17화부터 권력 역전으로, 30화부터 조사극으로 축이 두 번 바뀝니다. 새 사건과 새 장소를 계속 발명해야 회차가 차기 때문입니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="96" customHeight="1">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>이유 — 집필이 오히려 쉬워집니다</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="inlineStr">
+        <is>
+          <t>속마음이 열리면 사건 하나로 여러 화를 갈 수 있습니다. 레퍼런스 《욕망의 질주》는 차 뒷좌석 한 자리에서 15화를 가고, 사건 하나당 VO가 평균 15문장입니다. 새 방을 열지 않아도, 새 인물을 넣지 않아도 회차가 찹니다. 속마음을 막아 두면 매 화 새 사건을 만들어야 해서 집필이 훨씬 까다로워집니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="96" customHeight="1">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>이유 — 남성향 쿠거의 상품</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>남자 시청자는 남자 주인공 마음은 별로 안 궁금해도 여자 마음은 궁금합니다. '이 나이 많은 여자가 나를 원한다'가 확인되는 순간이 이 장르의 쾌감입니다. 다이앤의 속마음은 부수 요소가 아니라 파는 물건입니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="96" customHeight="1">
+      <c r="A6" s="9" t="inlineStr"/>
+      <c r="B6" s="9" t="inlineStr"/>
+    </row>
+    <row r="7" ht="96" customHeight="1">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>■ ★VO 개방 시차 — 둘을 같이 열지 않습니다</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr"/>
+    </row>
+    <row r="8" ht="96" customHeight="1">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>콜 = 1화부터</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>콜의 속마음은 1화부터 전부 열려 있습니다. 시청자는 콜에 얹혀서 봅니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="96" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>다이앤 = 6화부터</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>다이앤의 속은 1~5화 동안 완전히 닫아 둡니다. 화면으로는 보여주되(2화 밤 여덟 시 소파에 혼자 남는 컷) VO를 안 붙입니다. 이 여자가 무슨 생각인지 모르는 채로 첫 밤을 넘깁니다.
+★6화 욕실에서 처음 열립니다. 짧게, 결핍만 — '오래 참았다.' '이 나이에 이러고 있다.' 콜은 그 얼굴을 못 보고 시청자만 봅니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="96" customHeight="1">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>첫 만남 회상도 5화 차</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>콜의 첫 목격 = 3화 / 다이앤의 첫 목격 = 8화.
+같은 날 같은 현관을 두 번 쓰되 5화를 띄웁니다. 교차점은 콜이 재킷 앞자락을 급히 내려 잡는 손 하나입니다.
+★8화(무료 마지막)에서 다이앤이 한 줄로 회수합니다 — "이 년 전에 우리 집 현관에서, 너 재킷 왜 붙잡고 있었어?" … "그때부터 알고 있었어."</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="96" customHeight="1">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>왜 시차를 두나</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>둘을 같이 열면 첫 화에 답이 다 나와 버립니다. 시차를 두면 ①1~5화는 '이 여자 속을 모르겠다'가 긴장이 되고 ②6화에서 열리는 순간이 그 자체로 훅이 되며 ③8화 회수가 무료 마지막 화의 결제 카드가 됩니다. 카드를 세 번 나눠 씁니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="96" customHeight="1">
+      <c r="A12" s="9" t="inlineStr"/>
+      <c r="B12" s="9" t="inlineStr"/>
+    </row>
+    <row r="13" ht="96" customHeight="1">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>■ 무엇을 쓰는가</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr"/>
+    </row>
+    <row r="14" ht="96" customHeight="1">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>콜 VO — 3종만</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>① 흥분(몸의 반응) — '심장이 뛴다.' '또 선다.' '온몸이 굳는다.'
+② 사실관계 — '손 대면 끝이라고 했다.' '거실에 장인 있다.' '벽 하나다.'
+③ 계획 — '지금 다리 빼면 다시는 안 올라온다.' '오늘 밤 문 안 잠근다.'
+금지 — 자기평가('싫지는 않다'), 쿨한 척('색다른데?'), 감상, 멋부린 대구.
+규격 = 현재형·반말·파편. 평균 10자 안쪽. 문장을 완성하지 않습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="96" customHeight="1">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>다이앤 VO — 4종</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>① 결핍 — '나는 지금이 제일 셀 때인데.' '남편은 삼 년째 안 한다.'
+② 소유욕 — '가질 수도 있겠구나.' '내 것이라고 써 놓는 거다.'
+③ 위험을 아는 것 — '내 딸이 벽 하나 뒤에 있다.' '그래서 오늘이 제일 좋다.'
+④ 관찰 — '이 애는 아직 자기가 뭘 원하는지도 모른다.' '내가 알려 주면 된다.'
+규격 = 콜과 다르게 문장을 완성해도 됩니다. 나이와 여유의 차이를 레지스터로 냅니다. 다만 멋부린 문장·비유는 금지.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="96" customHeight="1">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>주변인물</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>★에이바·로사·하워드의 속마음은 절대 금지. 그들의 의심은 직접 발화(대사)로만 나옵니다.
+삭제 대상 지문 = '골똘히 생각에 잠긴다'(30화) / '그냥 사이가 좋을 뿐이야'(31화) / '답답한 마음'(37화) / '찜찜한 얼굴'(38화) / '의아함을 느낀다'(41화) / '찜찜한 표정'(42화) / '각자의 의심으로 불편한 공기'(45화)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="96" customHeight="1">
+      <c r="A17" s="9" t="inlineStr"/>
+      <c r="B17" s="9" t="inlineStr"/>
+    </row>
+    <row r="18" ht="96" customHeight="1">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>■ 첫 만남 — 이 작품의 출발점</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr"/>
+    </row>
+    <row r="19" ht="96" customHeight="1">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>방향 전환</t>
+        </is>
+      </c>
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>★'다이앤이 유혹했다'가 아닙니다. '콜이 처음 본 순간 이미 짜릿했다'입니다.
+지금 원고는 3화 플래시백을 '지난 몇 주간 다이앤의 은근한 유혹'으로 처리하는데, 그러면 콜은 당한 사람이 되고 배덕이 얕아집니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="96" customHeight="1">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>콜 쪽 (3화)</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>그녀의 입술, 목덜미, 풍만한 몸, 몸짓, 요염한 미소, 은근한 향. 어떤 여자에게서도 — 심지어 결혼할 에이바에게서도 — 느껴 본 적 없는 흥분. 심장이 맥박치고, 온몸이 긴장하고, 혈관이 팽창하고, 그곳이 빳빳해집니다. 장모 될 사람 앞에서.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="96" customHeight="1">
+      <c r="A21" s="10" t="inlineStr">
+        <is>
+          <t>다이앤 쪽 (8화)</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>성욕이 강하고 한창 더 강해질 시기인데 남편은 시들합니다. 발기도 안 되고 섹스에 무심합니다. 몸은 계속 달아오르는데 어쩌지를 못합니다.
+그 와중에 딸이 남자를 데려옵니다. 젊고 탄탄한 몸을 보고 — 딸이 부러웠습니다. 그러다 생각합니다. 어쩌면 내가 가질 수 있지 않을까.
+근거는 그날 그의 눈빛, 표정, 그리고 부풀어 있던 그의 고간입니다. 엄마뻘인 나를 보고 강하게 흥분했다는 것을 그녀는 알아봤습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="96" customHeight="1">
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>AIGC 주의</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>'부풀어 있던 고간'은 직접 그리지 않습니다. 재킷을 내려 잡는 손, 급히 돌아서는 몸, 그걸 따라가는 다이앤의 시선 — 세 컷으로 나눠서 전달합니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="96" customHeight="1">
+      <c r="A23" s="9" t="inlineStr"/>
+      <c r="B23" s="9" t="inlineStr"/>
+    </row>
+    <row r="24" ht="96" customHeight="1">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>■ 의심 비트에 대하여</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="inlineStr"/>
+    </row>
+    <row r="25" ht="96" customHeight="1">
+      <c r="A25" s="10" t="inlineStr">
+        <is>
+          <t>의심은 연료입니다</t>
+        </is>
+      </c>
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>주변인물의 의심은 그 자체가 이야기가 아니라, 두 사람을 더 달아오르게 하고 선을 더 넘게 만드는 연료입니다. 지금 원고는 30~46화에서 주변인물이 단서를 하나씩 수집하는 내용이 17화 가까이 이어져, 다이앤과 콜보다 조사하는 사람들이 주인공이 됩니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="96" customHeight="1">
+      <c r="A26" s="10" t="inlineStr">
+        <is>
+          <t>숫자</t>
+        </is>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>의심(직접 발화 추궁) 17화 → 3화(36화 목의 자국 / 39화 코롱 / 41화 서재).
+들킬랑말랑 8건 → 19건.
+나머지 회차는 두 사람의 심리와 야한 장면으로 채웁니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="96" customHeight="1">
+      <c r="A27" s="10" t="inlineStr">
+        <is>
+          <t>채워야 할 것</t>
+        </is>
+      </c>
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>빠져드는 쾌감 · 배덕감 · 배신을 저지르고 있다는 죄책감 · 그러나 그마저 조미료가 되는 정신적 쾌감 · 육체적 쾌감.
+배치 = 4화(배덕 점화) → 7화(죄책감이 조미료로) → 17화(죄책감 언어화) → 26화(배신 자각) → 29화(표시를 남기는 쾌감) → 35화(제일 진하고, 그게 다시 연료) → 47화</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -587,7 +899,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="150" customHeight="1">
+    <row r="3" ht="280" customHeight="1">
       <c r="A3" s="2" t="n">
         <v>2</v>
       </c>
@@ -610,16 +922,19 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>#3 뒤에 씬 추가 — #3-1 거실 / 밤 8시. 하워드가 약을 삼키고 "먼저 자겠네" 하고 올라간다. 다이앤이 소파에 혼자 남는다. TV를 끄지 않고 그냥 앉아 있다. 위층에서 문 닫히는 소리. ※'왜 하필 사위인가'의 답이 현재 작품에 없다. 이 한 컷이 다이앤의 결핍을 깐다.</t>
+          <t>#3 뒤에 씬 추가.
+★#3-1 거실 / 밤  여덟 시. 하워드가 약을 삼키고 "먼저 자겠네" 하고 올라간다. 다이앤이 소파에 혼자 남는다. TV를 끄지 않고 그냥 앉아 있다. 위층에서 문 닫히는 소리. 다이앤이 가운 자락을 무릎 위에서 만지작거리다 손을 뗀다. 한참 그러고 있는다.
+※'왜 하필 사위인가'의 답을 여기서 깐다. 단 ★VO는 아직 안 붙인다 — 화면으로만 보여주고 다이앤의 속은 6화까지 닫아 둔다(아래 'VO 개방 시차' 참조). 보여주고 말 안 하는 게 이 구간의 긴장이다.</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>다이앤(VO) '저 사람은 여덟 시면 끝난다.' / '나는 안 끝났는데.'  ·  콜 '삼 주다.' / '저 여자랑 둘이.'</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="150" customHeight="1">
+          <t>콜만. '삼 주다.' / '저 여자랑 둘이.'
+★다이앤 VO 없음 — 의도적으로 닫아 둔 구간.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="280" customHeight="1">
       <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
@@ -640,17 +955,32 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>발 자극 그대로 유지. ①플래시백 교체 — '지난 몇 주간 다이앤의 유혹'이 아니라 '콜이 이 년 전부터 다이앤을 봐 온 것'(첫 인사에서 안 놓던 손 / 결혼식장 첫 줄에서 다리를 바꿔 꼬던 것 / 신부 입장 중에 하객석을 보던 콜의 눈). ②VO 교체.</t>
+          <t>★플래시백 전면 교체 — '지난 몇 주간 다이앤이 유혹했다'가 아니라 '콜이 처음 본 순간 이미 짜릿했다'로. 발 자극은 그대로 유지.
+★#5-1 (플래시) 저택 현관 / 이 년 전 여름  딸이 남자를 데려온 날. 콜의 시점.
+문이 열린다. 민소매 원피스. 올려 묶은 머리, 목덜미에 땀으로 붙은 잔머리. 맨발에 슬리퍼.
+카메라가 콜의 시선을 그대로 따라간다 — 입술, 목덜미, 쇄골, 가슴에서 허리로 내려가는 천의 선, 돌아설 때의 걸음.
+악수. 끝났는데 손이 안 풀린다. 엄지가 그의 손등을 한 번 쓸고 놓는다.
+그녀가 웃는다. 눈꼬리가 내려간다. 앞서 들어가는 등이 깊게 파여 있다. 지나갈 때 향이 남는다.
+★콜이 재킷 앞자락을 급히 내려 잡는다.
+※재킷을 잡는 손이 이 작품의 씨앗이다. 8화에서 다이앤 쪽 시점으로 다시 나오고, 대사로 회수된다.</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>★콜은 유혹당하기 전에 이미 유혹돼 있던 남자.
-콜 '두 달 전부터 이 여자 생각하고 잤다.' / '지금 다리 빼면 다시는 안 올라온다.' / '안 뺀다.'</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="150" customHeight="1">
+          <t>★콜 심리 개방 정점. 유혹당하기 전에 이미 유혹돼 있던 남자.
+콜 '심장이 뛴다.'
+'온몸이 굳는다.'
+'무슨 냄새지, 이거.'
+'에이바한테서도 이런 적 없다.'
+'결혼할 여자한테서도 없었다.'
+'지금 이러면 안 되는데.'
+'섰다.'
+'장모 될 사람 앞에서.'
+(현재) '두 달 전부터 이 여자 생각하고 잤다.' / '지금 다리 빼면 다시는 안 올라온다.' / '안 뺀다.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="280" customHeight="1">
       <c r="A5" s="2" t="n">
         <v>4</v>
       </c>
@@ -671,13 +1001,19 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>규칙 선언 그대로. 앞에 한 줄 추가 — 콜이 달려들 때 다이앤 "이러면 안 돼. 넌 내 딸 남편이야." 그러면서 손은 콜의 셔츠를 안 놓는다. ※이 낙차가 작품 전체의 엔진인데 현재 한 번도 없다.</t>
+          <t>규칙 선언 그대로. 한 줄 추가 — 콜이 달려들 때 다이앤 "이러면 안 돼. 넌 내 딸 남편이야." 그러면서 손은 콜의 셔츠를 안 놓는다.
+※이 낙차가 작품 전체의 엔진인데 현재 한 번도 없다.
+※★다이앤 VO 여전히 없음. 이 여자가 무슨 생각인지 모르는 채로 4~5화를 끌고 간다.</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>★배덕이 처음 켜지는 화.
-다이앤(VO) '이 애가 내 딸이랑 자는 방이 복도 끝이다.' / '그걸 알면서 문을 열었다.'  ·  콜 '머리 젖었다.' / '나 올 줄 알았나.'</t>
+          <t>★배덕이 처음 켜지는 화. 콜만.
+콜 '머리 젖었다.'
+'방금 씻었네.'
+'나 올 줄 알았나.'
+'모르겠다. 이 여자 속을.'
+★다이앤 VO 없음.</t>
         </is>
       </c>
     </row>
@@ -707,12 +1043,12 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>콜 '손 대면 끝이라고 했다.' / '그래서 안 댄다.' / '미치겠네.' / '이 여자가 내 장모다.' / '그 생각 하니까 더 된다.'
-다이앤(VO) '아직 아무것도 모르는 얼굴이네.'</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="150" customHeight="1">
+          <t>콜만. '손 대면 끝이라고 했다.' / '그래서 안 댄다.' / '미치겠네.' / '이 여자가 내 장모다.' / '그 생각 하니까 더 된다.'
+★다이앤 VO 없음 — 다음 화에서 처음 열린다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="280" customHeight="1">
       <c r="A7" s="2" t="n">
         <v>6</v>
       </c>
@@ -733,13 +1069,18 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>그대로.</t>
+          <t>행위 그대로. ★이 화가 다이앤 속마음이 처음 열리는 지점이다.
+슬립째 샤워기 아래로 걸어 들어와 콜에게 몸을 붙이는 동안, 카메라가 다이앤의 얼굴에 한 번 머문다. 콜은 그 얼굴을 못 본다(눈이 감겨 있거나 등 뒤). 시청자만 본다.
+※1~5화는 콜 시점으로만 끌고 오다가 여기서 처음 다이앤 안쪽이 열린다. '이 여자도 원하고 있었다'가 확인되는 순간 자체가 훅이다.</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>콜 '옷 안 벗을 건가.' / '젖으니까 다 비친다.' / '손 못 쓴다.'
-다이앤(VO) '이 나이에 이런 걸 하고 있다.' / '오래 참았다.'</t>
+          <t>★다이앤 VO 최초 개방 — 짧게, 결핍만. 아직 첫 만남 얘기는 안 한다.
+다이앤(VO) '오래 참았다.'
+'이 나이에 이러고 있다.'
+'그런데 안 멈춰진다.'
+콜 '옷 안 벗을 건가.' / '젖으니까 다 비친다.' / '손 못 쓴다.'</t>
         </is>
       </c>
     </row>
@@ -775,7 +1116,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="150" customHeight="1">
+    <row r="9" ht="280" customHeight="1">
       <c r="A9" s="2" t="n">
         <v>8</v>
       </c>
@@ -796,12 +1137,30 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>【무료 마지막】 그대로. 대사 한 줄 — "상 받을 준비가 됐나 보네. 우리 강아지." ※모성이 겹쳐야 남성향 쿠거로 소구된다.</t>
+          <t>【무료 마지막】 행위 그대로. 두 가지 추가.
+①대사 — "상 받을 준비가 됐나 보네. 우리 강아지." (모성이 겹쳐야 남성향 쿠거로 소구된다)
+②★첫 만남 회수 — 브래지어를 풀기 직전에 다이앤이 묻는다.
+다이앤 "이 년 전에 우리 집 현관에서, 너 재킷 왜 붙잡고 있었어?"
+콜이 대답을 못 한다.
+다이앤 "그때부터 알고 있었어."
+★#10-1 (플래시) 저택 현관 / 이 년 전 여름 — 3화와 같은 날, 다이앤 시점.
+티셔츠 위로 드러난 어깨와 팔, 굵은 목, 셔츠가 당겨진 가슴. 인사를 하고 돌아서는 콜이 재킷 앞자락을 급히 내려 잡는다. 다이앤이 그 손을 본다. 그리고 그의 눈이 자기 목덜미에 멎어 있었다는 것도.
+※같은 컷을 3화(콜)와 8화(다이앤)로 두 번 쓴다. 5화 차이를 두고 반대편이 열리는 구조.
+※무료 마지막 화가 '첫 삽입 허락' + '그때부터 알고 있었어' 두 장으로 끝난다.</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>콜 '드디어.' / '버클이 안 풀린다.' / '손이 떨려서.'</t>
+          <t>★다이앤 첫 목격 전면 개방. 여기가 무료 구간 최대 카드.
+다이앤(VO) '남편은 삼 년째 안 한다.'
+'해 보려고 해도 안 된다.'
+'나는 지금이 제일 셀 때인데.'
+'그날 딸이 남자를 데려왔다. 젊고, 단단하고, 목이 굵었다.'
+'딸이 부러웠다.'
+'그런데 그 애가 나를 그렇게 봤다. 엄마뻘인 나를 보고.'
+'그날 알았다. 가질 수도 있겠구나.'
+'이 년 기다렸다.'
+콜 '드디어.' / '알고 있었대.' / '그럼 이 년 동안 저 여자도.' / '버클이 안 풀린다.'</t>
         </is>
       </c>
     </row>
@@ -2122,7 +2481,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2302,12 +2661,14 @@
     <row r="17" ht="44" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
         <is>
-          <t>다이앤 VO 개방</t>
+          <t>다이앤 VO 개방 (확정)</t>
         </is>
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>캐논 '속마음 폐쇄 · 어디까지 우연인지 끝까지 미확정'과 충돌. 이번 지시를 정본으로 올릴지 확인 필요 — 올리면 meta 갱신</t>
+          <t>★사용자 지시로 캐논 해제. 00_meta.md '다이앤 속마음 폐쇄 · 그녀 전용 내레이션 금지' 조항을 '두 사람 속마음 개방 · 단 개방 시차 5화'로 갱신 필요.
+사유 = 성행위만으로 50화를 채울 수 없고, 속마음이 열려야 사건 하나로 여러 화를 갈 수 있어 집필이 쉬워진다.
+시차 = 콜 1화 / 다이앤 6화. 첫 만남 회상은 콜 3화 / 다이앤 8화.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto commit (2026-08-21 20:01) — 1 changes
Claude Code 세션 종료 시 자동 커밋.

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/projects/18_while_my_wifes_away/18_while_my_wifes_away_w3_writer_table_actions.xlsx
+++ b/projects/18_while_my_wifes_away/18_while_my_wifes_away_w3_writer_table_actions.xlsx
@@ -518,7 +518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B27"/>
+  <dimension ref="A1:B29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -541,7 +541,7 @@
       </c>
       <c r="B2" s="9" t="inlineStr">
         <is>
-          <t>다이앤과 콜, 두 사람의 속마음(VO·감각 묘사)을 전면 개방합니다. 기존 기획안의 '다이앤 속마음 폐쇄' 조항은 이번 라운드로 해제합니다.</t>
+          <t>다이앤과 콜, 두 사람의 속마음(VO·감각 묘사)을 여는 방향으로 가려고 합니다. 처음 기획안에 있던 '다이앤 속마음 폐쇄' 조항은 이번에 저희 쪽에서 풀었습니다. 사정은 아래에 적어 두었습니다.</t>
         </is>
       </c>
     </row>
@@ -656,35 +656,35 @@
       </c>
       <c r="B13" s="9" t="inlineStr"/>
     </row>
-    <row r="14" ht="96" customHeight="1">
+    <row r="14" ht="230" customHeight="1">
       <c r="A14" s="10" t="inlineStr">
         <is>
-          <t>콜 VO — 3종만</t>
-        </is>
-      </c>
-      <c r="B14" s="9" t="inlineStr">
+          <t>VO는 자리에 따라 길이가 다릅니다</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>① 개방 VO (회상 · 첫 목격 · 결핍) — 긴 산문형.
+   완결된 문장으로 감각을 하나씩 쌓아 올리는 쪽이 맞습니다. 3화 콜 / 8화 다이앤이 여기 해당합니다. 레퍼런스 《욕망의 질주》 첫 VO도 이 형태입니다 — 'Every time the car hit a bump, my 18-year-old stepson's burning hand pushed another inch up under my skirt.'
+   처리표 3화·8화 칸에 참고안을 적어 두었습니다.
+② 현장 VO (행위 중 · 반응) — 파편형.
+   현재형·반말로, 문장을 완성하지 않는 쪽이 잘 붙습니다. '또 선다.' '벽 하나다.' '안 뺀다.' 이유나 결과를 붙이지 않고 반응만 남기면 됩니다.
+앞서 드린 '짧게' 요청은 ②를 두고 드린 말이었습니다. ①까지 짧게 가면 감각이 날아가니 거기서는 마음껏 늘려 주셔도 됩니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="140" customHeight="1">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>콜의 VO는 이런 것들</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
         <is>
           <t>① 흥분(몸의 반응) — '심장이 뛴다.' '또 선다.' '온몸이 굳는다.'
 ② 사실관계 — '손 대면 끝이라고 했다.' '거실에 장인 있다.' '벽 하나다.'
 ③ 계획 — '지금 다리 빼면 다시는 안 올라온다.' '오늘 밤 문 안 잠근다.'
-금지 — 자기평가('싫지는 않다'), 쿨한 척('색다른데?'), 감상, 멋부린 대구.
-규격 = 현재형·반말·파편. 평균 10자 안쪽. 문장을 완성하지 않습니다.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="96" customHeight="1">
-      <c r="A15" s="10" t="inlineStr">
-        <is>
-          <t>다이앤 VO — 4종</t>
-        </is>
-      </c>
-      <c r="B15" s="9" t="inlineStr">
-        <is>
-          <t>① 결핍 — '나는 지금이 제일 셀 때인데.' '남편은 삼 년째 안 한다.'
-② 소유욕 — '가질 수도 있겠구나.' '내 것이라고 써 놓는 거다.'
-③ 위험을 아는 것 — '내 딸이 벽 하나 뒤에 있다.' '그래서 오늘이 제일 좋다.'
-④ 관찰 — '이 애는 아직 자기가 뭘 원하는지도 모른다.' '내가 알려 주면 된다.'
-규격 = 콜과 다르게 문장을 완성해도 됩니다. 나이와 여유의 차이를 레지스터로 냅니다. 다만 멋부린 문장·비유는 금지.</t>
+자기평가('싫지는 않다')나 쿨한 척('색다른데?')으로 가면 콜이 이미 다 아는 남자처럼 보여서, 흥분·사실·계획 셋 안에서 잡아 주시면 좋겠습니다.</t>
         </is>
       </c>
     </row>
@@ -696,8 +696,8 @@
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>★에이바·로사·하워드의 속마음은 절대 금지. 그들의 의심은 직접 발화(대사)로만 나옵니다.
-삭제 대상 지문 = '골똘히 생각에 잠긴다'(30화) / '그냥 사이가 좋을 뿐이야'(31화) / '답답한 마음'(37화) / '찜찜한 얼굴'(38화) / '의아함을 느낀다'(41화) / '찜찜한 표정'(42화) / '각자의 의심으로 불편한 공기'(45화)</t>
+          <t>다만 에이바·로사·하워드의 속마음은 안 여는 쪽으로 부탁드립니다. 그들의 의심은 대사로만 나오면 좋겠습니다.
+지금 원고에서 이 계열에 해당하는 지문 — '골똘히 생각에 잠긴다'(30화) / '그냥 사이가 좋을 뿐이야'(31화) / '답답한 마음'(37화) / '찜찜한 얼굴'(38화) / '의아함을 느낀다'(41화) / '찜찜한 표정'(42화) / '각자의 의심으로 불편한 공기'(45화). 대사나 행동으로 바꿔 주시면 시점이 정리됩니다.</t>
         </is>
       </c>
     </row>
@@ -721,8 +721,8 @@
       </c>
       <c r="B19" s="11" t="inlineStr">
         <is>
-          <t>★'다이앤이 유혹했다'가 아닙니다. '콜이 처음 본 순간 이미 짜릿했다'입니다.
-지금 원고는 3화 플래시백을 '지난 몇 주간 다이앤의 은근한 유혹'으로 처리하는데, 그러면 콜은 당한 사람이 되고 배덕이 얕아집니다.</t>
+          <t>첫 만남을 '다이앤이 유혹했다'가 아니라 '콜이 처음 본 순간 이미 짜릿했다'로 잡아 주시면 좋겠습니다.
+지금 3화 플래시백이 '지난 몇 주간 다이앤의 은근한 유혹'으로 되어 있는데, 그러면 콜이 당한 사람이 되어서 배덕감이 조금 얕아지는 것 같습니다.</t>
         </is>
       </c>
     </row>
@@ -760,7 +760,7 @@
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>'부풀어 있던 고간'은 직접 그리지 않습니다. 재킷을 내려 잡는 손, 급히 돌아서는 몸, 그걸 따라가는 다이앤의 시선 — 세 컷으로 나눠서 전달합니다.</t>
+          <t>'부풀어 오른 고간'은 AI 영상으로 직접 잡기가 어렵습니다. 재킷을 내려 잡는 손 / 급히 돌아서는 몸 / 그걸 따라가는 다이앤의 시선, 세 컷으로 나눠 주시면 전달됩니다.</t>
         </is>
       </c>
     </row>
@@ -784,7 +784,8 @@
       </c>
       <c r="B25" s="11" t="inlineStr">
         <is>
-          <t>주변인물의 의심은 그 자체가 이야기가 아니라, 두 사람을 더 달아오르게 하고 선을 더 넘게 만드는 연료입니다. 지금 원고는 30~46화에서 주변인물이 단서를 하나씩 수집하는 내용이 17화 가까이 이어져, 다이앤과 콜보다 조사하는 사람들이 주인공이 됩니다.</t>
+          <t>주변인물의 의심은 그 자체가 이야기라기보다, 두 사람을 더 달아오르게 하고 선을 더 넘게 만드는 연료 쪽으로 써 주시면 좋겠습니다.
+지금은 30~46화에서 주변인물이 단서를 하나씩 모으는 내용이 17화 가까이 이어져서, 다이앤과 콜보다 조사하는 사람들이 앞에 서는 느낌입니다.</t>
         </is>
       </c>
     </row>
@@ -812,6 +813,35 @@
         <is>
           <t>빠져드는 쾌감 · 배덕감 · 배신을 저지르고 있다는 죄책감 · 그러나 그마저 조미료가 되는 정신적 쾌감 · 육체적 쾌감.
 배치 = 4화(배덕 점화) → 7화(죄책감이 조미료로) → 17화(죄책감 언어화) → 26화(배신 자각) → 29화(표시를 남기는 쾌감) → 35화(제일 진하고, 그게 다시 연료) → 47화</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="150" customHeight="1">
+      <c r="A28" s="10" t="inlineStr">
+        <is>
+          <t>다이앤의 VO는 이런 것들</t>
+        </is>
+      </c>
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>① 결핍 — '욕망이 가장 뜨겁게 불타오를 나이건만, 남편은 이미 시들해진 지 오래였다.'
+② 소유욕 — '어쩌면... 내가 저 아이를 가질 수 있지 않을까?'
+③ 위험을 아는 것 — '내 딸이 벽 하나 뒤에 있다. 그래서 오늘이 제일 좋다.'
+④ 관찰 — '이 애는 아직 자기가 뭘 원하는지도 모른다.'
+콜보다 문장이 길고 완결되는 쪽이 좋습니다. 나이와 여유의 차이가 문장 길이로 나면 두 사람이 잘 갈립니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="150" customHeight="1">
+      <c r="A29" s="10" t="inlineStr">
+        <is>
+          <t>참고안 위치</t>
+        </is>
+      </c>
+      <c r="B29" s="11" t="inlineStr">
+        <is>
+          <t>콜 첫 목격 VO = 처리표 3화 칸 / 다이앤 첫 목격 VO = 처리표 8화 칸.
+두 칸 모두 참고용 예시입니다. 그대로 쓰셔도 되고 작가님 문장으로 다시 쓰셔도 됩니다.</t>
         </is>
       </c>
     </row>
@@ -934,7 +964,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="280" customHeight="1">
+    <row r="4" ht="430" customHeight="1">
       <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
@@ -967,16 +997,12 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>★콜 심리 개방 정점. 유혹당하기 전에 이미 유혹돼 있던 남자.
-콜 '심장이 뛴다.'
-'온몸이 굳는다.'
-'무슨 냄새지, 이거.'
-'에이바한테서도 이런 적 없다.'
-'결혼할 여자한테서도 없었다.'
-'지금 이러면 안 되는데.'
-'섰다.'
-'장모 될 사람 앞에서.'
-(현재) '두 달 전부터 이 여자 생각하고 잤다.' / '지금 다리 빼면 다시는 안 올라온다.' / '안 뺀다.'</t>
+          <t>이 정도 결의 VO를 생각하고 있습니다. 참고용으로 적어 두니 편하게 보시고, 작가님 문장으로 다시 쓰셔도 좋습니다. 밀도와 감각의 눈금만 이만큼 나와 주면 좋겠습니다.
+【콜 VO 참고안 / #5-1 플래시 위에 얹음】
+다이앤을 처음 본 순간, 온몸의 피가 역류하는 것 같은 짜릿한 전율이 뇌리를 덮쳤다. 붉고 촉촉한 입술, 선이 고운 목덜미, 옷감 너머로 감출 수 없는 풍만한 몸매와 은밀한 몸짓, 요염한 미소, 그리고 코끝을 스치는 은근한 향기까지. 그 어떤 여자에게서도, 심지어 내 아내가 될 에이바에게서조차 단 한 번도 느껴보지 못한 강렬한 흥분이었다. 심장이 터질 듯 맥박 치고 온몸의 신경이 바짝 긴장했다. 혈관이 팽창하며 피가 아래로 솟구쳤고, 바지 속이 한없이 빳빳하게 죄어오는 감각에 숨이 턱 막혔다.
+붙는 자리는 문이 열리고 다이앤이 나타나는 컷부터 콜이 재킷 앞자락을 내려 잡는 컷까지입니다. 지문은 그 사이에 입술 → 목덜미 → 쇄골 → 허리선 → 돌아서는 걸음 순으로 카메라를 움직이면 VO와 붙습니다.
+【현재로 돌아온 뒤 · 짧은 파편형】
+콜 '두 달 전부터 이 여자 생각하고 잤다.' / '지금 다리 빼면 다시는 안 올라온다.' / '안 뺀다.'</t>
         </is>
       </c>
     </row>
@@ -1116,7 +1142,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="280" customHeight="1">
+    <row r="9" ht="430" customHeight="1">
       <c r="A9" s="2" t="n">
         <v>8</v>
       </c>
@@ -1151,15 +1177,11 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>★다이앤 첫 목격 전면 개방. 여기가 무료 구간 최대 카드.
-다이앤(VO) '남편은 삼 년째 안 한다.'
-'해 보려고 해도 안 된다.'
-'나는 지금이 제일 셀 때인데.'
-'그날 딸이 남자를 데려왔다. 젊고, 단단하고, 목이 굵었다.'
-'딸이 부러웠다.'
-'그런데 그 애가 나를 그렇게 봤다. 엄마뻘인 나를 보고.'
-'그날 알았다. 가질 수도 있겠구나.'
-'이 년 기다렸다.'
+          <t>무료 마지막 화라 여기가 제일 큰 카드입니다. 아래는 참고안이고, 작가님 문장으로 다시 쓰셔도 좋습니다. 결핍과 첫 목격이 한 덩어리로 나오는 것만 지켜지면 됩니다.
+【다이앤 VO 참고안 / #10-1 플래시 위에 얹음】
+몸이 감당하기 힘들 정도로 달아올라 있던 시기였다. 욕망이 가장 뜨겁게 불타오를 나이건만, 남편은 이미 시들해진 지 오래였다. 발기조차 되지 않는 무심한 몸을 곁에 두고 매일 밤 홀로 속을 끓여야 했던 나날들. 그러던 중 딸아이가 제 연인이라며 콜을 데려왔다. 젊고 탄탄한 그의 몸매를 마주한 순간, 솔직히 딸아이가 부러울 지경이었다. 하지만 그 부러움은 순식간에 은밀한 욕심으로 바뀌었다. '어쩌면... 내가 저 아이를 가질 수 있지 않을까?' 나를 처음 바라보던 그 애의 흔들리던 눈빛, 굳어버린 표정, 그리고 바지 위로 묵직하게 부풀어 오른 고간. 엄마뻘인 나를 보고 주체할 수 없이 강하게 흥분했음을, 나는 한눈에 알아채고 말았다.
+'바지 위로 묵직하게 부풀어 오른 고간'은 화면에 직접 잡기 어려운 컷이라, 재킷을 내려 잡는 손 → 급히 돌아서는 몸 → 그걸 따라가는 다이앤의 시선, 세 컷으로 나눠 주시면 전달됩니다.
+【현재 · 짧은 파편형】
 콜 '드디어.' / '알고 있었대.' / '그럼 이 년 동안 저 여자도.' / '버클이 안 풀린다.'</t>
         </is>
       </c>

</xml_diff>